<commit_message>
fix: finalize capstone alignment and reporting contracts
</commit_message>
<xml_diff>
--- a/sample_data/future_import_template.xlsx
+++ b/sample_data/future_import_template.xlsx
@@ -26,12 +26,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color theme="3"/>
-      <sz val="15"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -51,26 +46,23 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-    <cellStyle name="Headline 1" xfId="1" builtinId="16" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -439,7 +431,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CUSTOMER NAME</t>
+          <t>ACCOUNT NAMES</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">

</xml_diff>